<commit_message>
GATEWAY 1.0: aggiunti test OK CT24/CT25 (checklist 448, 449) con report 234-235, PDF e righe report-checklist.
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/GATEWAY/S1111TREINFORMATIONTECHNOLOGYXX/3IT/TREINFORMATIONTECHNOLOGYXX/1.0/report-checklist.xlsx
+++ b/GATEWAY/S1111TREINFORMATIONTECHNOLOGYXX/3IT/TREINFORMATIONTECHNOLOGYXX/1.0/report-checklist.xlsx
@@ -1085,7 +1085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W28"/>
+  <dimension ref="A1:W30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="11.453125" customWidth="1" style="50" min="1" max="1"/>
@@ -3057,7 +3057,7 @@
     </row>
     <row r="26" ht="11.15" customHeight="1" s="50" thickBot="1">
       <c r="A26" t="n">
-        <v>461</v>
+        <v>448</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -3071,29 +3071,29 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>VALIDAZIONE_CDA2_RSA_CT26_KO</t>
+          <t>VALIDAZIONE_CDA2_RSA_CT24</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation" al fine di testare la gestione degli errori terminologici sui Dati (status code 400), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway. 
-I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 26" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
+          <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation", al fine di una futura pubblicazione, con esito positivo (status code 201), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+Il Documento CDA2 Referto Specialistica Ambulatoriale dovrà essere composto in modo da risultare valido dal punto di vista sintattico, semantico, terminologico. I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso dalla sezione "CASO DI TEST 24" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_OK" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
       <c r="F26" s="90" t="n">
         <v>46123</v>
       </c>
       <c r="G26" s="91" t="n">
-        <v>0.7865277777777778</v>
+        <v>0.8332638888888889</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>cc1e2f08e48204678b2c2a8ee17ba702</t>
+          <t>2425e44cb99726aa3421420208de2cd9</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.d0c5f604a969a37e4498da27d3165fc66898496385879df1fe5f06e9f83d374e.894c96ffa6^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.d1cadaafd3c35cea0f35a0f361d86d08e6e4607e5f2ce8068fbf64030202acc2.f094f52607^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -3103,22 +3103,22 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>HTTP 422 — validazione rifiutata. [ERRORE-b24| Sezione Storia Clinica: l'elemento entry/observation/code deve avere l'attributo @code='75326-9' e l'attributo @codeSystem='2.16.840.1.113883.6.1'],[ERRORE-b26| Sezione Storia Clinica: l'elemento entry/observation/effectiveTime deve essere presente e deve avere l'elemento 'low' valorizzato],[ERRORE-b20| Il codice '48765-2' non è corret</t>
+          <t>HTTP 201 — validazione documento superata (CASO TEST 24 / checklist 448).</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -3128,12 +3128,12 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Correzione dati/CDA e nuovo invio validazione Gateway.</t>
+          <t>Non applicabile (esito positivo).</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
@@ -3148,18 +3148,18 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>MedSend. PDF in FILES: CT461_RSA_VALIDATION_REPORT_229_FSE_READY.PDF.</t>
+          <t>MedSend. PDF in FILES: CT448_RSA_VALIDATION_REPORT_234_FSE_READY.PDF. Report MedSend #234.</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="27" ht="11.15" customHeight="1" s="50" thickBot="1">
       <c r="A27" t="n">
-        <v>468</v>
+        <v>449</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -3173,29 +3173,29 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>VALIDAZIONE_CDA2_RSA_CT27_KO</t>
+          <t>VALIDAZIONE_CDA2_RSA_CT25</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation" al fine di testare la gestione degli errori sintattici sui Dati (status code 400), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
-I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 27" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
+          <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation", al fine di una futura pubblicazione, con esito positivo (status code 201), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+Il Documento CDA2 Referto Specialistica Ambulatoriale dovrà essere composto in modo da risultare valido dal punto di vista sintattico, semantico, terminologico. I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso dalla sezione "CASO DI TEST 25" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_OK" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
       <c r="F27" s="90" t="n">
         <v>46123</v>
       </c>
       <c r="G27" s="91" t="n">
-        <v>0.7865393518518519</v>
+        <v>0.833275462962963</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>c75270d4ea3304a9413f5d27021d99cc</t>
+          <t>a9310b244e9ad4ab799c797803bd396c</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.e10fa16d17faf284bdc4bbde862f6b3c7c984961e76fc245fe6a8259d4244553.d7bfb4f1ff^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.51584702dea24abf297a5f6b36feb0b908423edaab535df44d0c8dbceb693d7a.31ae1ee8e2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -3205,22 +3205,22 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>HTTP 400 — validazione rifiutata. ERROR: -1,-1 cvc-complex-type.2.4.a: Invalid content was found starting with element '{"urn:hl7-org:v3":languageCode}'. One of '{"urn:hl7-org:v3":confidentialityCode}' is expected.</t>
+          <t>HTTP 201 — validazione documento superata (CASO TEST 25 / checklist 449).</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -3230,12 +3230,12 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Correzione dati/CDA e nuovo invio validazione Gateway.</t>
+          <t>Non applicabile (esito positivo).</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
@@ -3250,119 +3250,321 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>MedSend. PDF in FILES: CT468_RSA_VALIDATION_REPORT_230_FSE_READY.PDF.</t>
+          <t>MedSend. PDF in FILES: CT449_RSA_VALIDATION_REPORT_235_FSE_READY.PDF. Report MedSend #235.</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="28" ht="11.15" customHeight="1" s="50" thickBot="1">
       <c r="A28" t="n">
+        <v>461</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>VALIDAZIONE</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>RSA</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>VALIDAZIONE_CDA2_RSA_CT26_KO</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation" al fine di testare la gestione degli errori terminologici sui Dati (status code 400), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway. 
+I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 26" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
+        </is>
+      </c>
+      <c r="F28" s="90" t="n">
+        <v>46123</v>
+      </c>
+      <c r="G28" s="91" t="n">
+        <v>0.7865277777777778</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>cc1e2f08e48204678b2c2a8ee17ba702</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.d0c5f604a969a37e4498da27d3165fc66898496385879df1fe5f06e9f83d374e.894c96ffa6^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>HTTP 422 — validazione rifiutata. [ERRORE-b24| Sezione Storia Clinica: l'elemento entry/observation/code deve avere l'attributo @code='75326-9' e l'attributo @codeSystem='2.16.840.1.113883.6.1'],[ERRORE-b26| Sezione Storia Clinica: l'elemento entry/observation/effectiveTime deve essere presente e deve avere l'elemento 'low' valorizzato],[ERRORE-b20| Il codice '48765-2' non è corret</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Correzione dati/CDA e nuovo invio validazione Gateway.</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Superato</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>MedSend. PDF in FILES: CT461_RSA_VALIDATION_REPORT_229_FSE_READY.PDF.</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="11.15" customHeight="1" s="50" thickBot="1">
+      <c r="A29" t="n">
+        <v>468</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>VALIDAZIONE</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>RSA</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>VALIDAZIONE_CDA2_RSA_CT27_KO</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation" al fine di testare la gestione degli errori sintattici sui Dati (status code 400), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 27" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
+        </is>
+      </c>
+      <c r="F29" s="90" t="n">
+        <v>46123</v>
+      </c>
+      <c r="G29" s="91" t="n">
+        <v>0.7865393518518519</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>c75270d4ea3304a9413f5d27021d99cc</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.e10fa16d17faf284bdc4bbde862f6b3c7c984961e76fc245fe6a8259d4244553.d7bfb4f1ff^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>HTTP 400 — validazione rifiutata. ERROR: -1,-1 cvc-complex-type.2.4.a: Invalid content was found starting with element '{"urn:hl7-org:v3":languageCode}'. One of '{"urn:hl7-org:v3":confidentialityCode}' is expected.</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Correzione dati/CDA e nuovo invio validazione Gateway.</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Superato</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>MedSend. PDF in FILES: CT468_RSA_VALIDATION_REPORT_230_FSE_READY.PDF.</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="11.15" customHeight="1" s="50" thickBot="1">
+      <c r="A30" t="n">
         <v>475</v>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>VALIDAZIONE</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>RSA</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>VALIDAZIONE_CDA2_RSA_CT28_KO</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation" al fine di testare la gestione degli errori terminologici sui Dati (status code 400), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway. 
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 28" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
         </is>
       </c>
-      <c r="F28" s="90" t="n">
+      <c r="F30" s="90" t="n">
         <v>46123</v>
       </c>
-      <c r="G28" s="91" t="n">
+      <c r="G30" s="91" t="n">
         <v>0.7865393518518519</v>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>89015c45a5d4d6bbd3463789ace1737c</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>2.16.840.1.113883.2.9.2.120.4.4.cc04145ef5192976dfb48039aa011f6f1da17487a5e99fa54472b4a27f0cf1b9.553ad3155c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
         <is>
           <t>HTTP 422 — validazione rifiutata. [ERRORE-b20| Il codice '48765-2' non è corretto. La sezione deve essere valorizzata con uno dei seguenti codici:</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr">
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr">
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
         <is>
           <t>Correzione dati/CDA e nuovo invio validazione Gateway.</t>
         </is>
       </c>
-      <c r="T28" t="inlineStr">
+      <c r="T30" t="inlineStr">
         <is>
           <t>Superato</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr">
+      <c r="U30" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="V28" t="inlineStr">
+      <c r="V30" t="inlineStr">
         <is>
           <t>MedSend. PDF in FILES: CT475_RSA_VALIDATION_REPORT_231_FSE_READY.PDF.</t>
         </is>
       </c>
-      <c r="W28" t="inlineStr">
+      <c r="W30" t="inlineStr">
         <is>
           <t>KO</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="11.15" customHeight="1" s="50" thickBot="1"/>
-    <row r="30" ht="11.15" customHeight="1" s="50" thickBot="1"/>
     <row r="31" ht="11.15" customHeight="1" s="50" thickBot="1"/>
     <row r="32" ht="11.15" customHeight="1" s="50" thickBot="1"/>
     <row r="33" ht="11.15" customHeight="1" s="50" thickBot="1"/>

</xml_diff>